<commit_message>
EA-50 v2.1: enrichment complete — 117 named-seat rows (40 on-record + 77 enriched/verified, 4 wings); SPK removal 19-Oct verified live (Official Gazette, successor vacant); SA/GCC wing salvaged at iteration cap
</commit_message>
<xml_diff>
--- a/ChainSentry-EA50-Master-Targets-20261020.xlsx
+++ b/ChainSentry-EA50-Master-Targets-20261020.xlsx
@@ -6480,7 +6480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:I118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8339,100 +8339,100 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>SPK (Sermaye Piyasasi Kurulu / Capital Markets Board)</t>
+          <t>SAMA (Saudi Central Bank)</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Mahmut Sutcu</t>
+          <t>Ayed Al-Amroq</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Kurul Chairman (appointed 9 May 2026 | removed from office 19-20 Oct 2026, successor not yet named at time of research)</t>
+          <t>Governor</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr"/>
       <c r="G47" s="5" t="inlineStr"/>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>https://www.dunya.com (Dunya Gazetesi: "SPK Baskani Mahmut Sutcu ve KGK Baskani Ibrahim Omer Gonul gorevden alindi", 20 Oct 2026 | original appointment: A Haber 9 May 2026, tr.wikipedia.org/wiki/Sermaye_Piyasas%C4%B1_Kurumu)</t>
+          <t>https://news.google.com/rss/search?q=SAMA+governor+Saudi+Arabia</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
+          <t>ENRICHED 2026-10-20 · 2026-10-19</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>SPK (Sermaye Piyasasi Kurulu)</t>
+          <t>SAMA (Saudi Central Bank)</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>(position-only)</t>
+          <t>Abdulaziz Abanmi</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Head of digital-assets / crypto licensing division (SPK oversees VASP licensing under Law 7518 | division head not publicly named)</t>
+          <t>Deputy Governor for Payments (oversees regulatory sandbox/fintech policy)</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr"/>
       <c r="G48" s="5" t="inlineStr"/>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>https://spk.gov.tr/hakkimizda/kurul-baskani</t>
+          <t>https://thefintechtimes.com/inside-samas-strategy-how-saudi-arabia-is-engineering-the-future-of-payments/</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
+          <t>ENRICHED 2026-10-20 · 2025-10-05</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>MASAK (Financial Crimes Investigation Board)</t>
+          <t>CMA Saudi Arabia</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Hasan Kaymak</t>
+          <t>Mazen Al-Sudairi</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>President of MASAK (appointed Feb 2024 | publicly active as MASAK head Oct 2026)</t>
+          <t>Chairman of the Capital Market Authority (appointed by royal decree)</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -8444,190 +8444,190 @@
       <c r="G49" s="5" t="inlineStr"/>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>https://www.aa.com.tr (Anadolu/AHaber 23 Feb 2024 | Anka Haber 14 Oct 2026 "MASAK Baskani Kaymak")</t>
+          <t>https://news.google.com/rss/search?q=Mazen+Al-Sudairi+CMA</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-14</t>
+          <t>ENRICHED 2026-10-20 · 2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>MASAK (Financial Crimes Investigation Board)</t>
+          <t>CMA Saudi Arabia</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>(position-only)</t>
+          <t>UNFILLED (position-only</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Uyum / compliance programme lead (AML compliance supervision directorate | individual not publicly named)</t>
+          <t>head of FinTech Permit/lab not publicly named)</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>Head of FinTech Permit &amp; innovation lab</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr"/>
       <c r="G50" s="5" t="inlineStr"/>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>https://www.masak.gov.tr</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
+          <t>ENRICHED 2026-10-20 · https://news.google.com/rss/search?q=%22Saudi+Capital+Market+Authority%22+chairman</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>BtcTurk</t>
+          <t>Saudi Financial Investigations Unit (SAFIU)</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Tevfik Kinik</t>
+          <t>UNFILLED (position-only</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>CEO of BtcTurk Group Companies (appointed Jan 2026)</t>
+          <t>head not identified in 2025-26 sources)</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>Head of SAFIU (AML/CFT FIU)</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr"/>
       <c r="G51" s="5" t="inlineStr"/>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>https://www.aa.com.tr (Anadolu Ajansi &amp; DHA 6 Jan 2026 "BtcTurk'te ust duzey atama" | Fortune Turkey)</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-01-06</t>
+          <t>ENRICHED 2026-10-20 · https://news.google.com/rss/search?q=SAFIU+Saudi+financial+investigations</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>BtcTurk</t>
+          <t>Alrajhi Bank</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Fatih Otluoglu</t>
+          <t>Waleed Al-Mogbel</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>CEO of BtcTurk Hisse (brokerage arm)</t>
+          <t>Group CEO (confirmed through 2025 best-CEO award</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>high</t>
+          <t xml:space="preserve"> 2026 results quoted via Abdullah Alrajhi - needs verification)</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr"/>
       <c r="G52" s="5" t="inlineStr"/>
       <c r="H52" s="5" t="inlineStr">
         <is>
-          <t>https://www.ekonomim.com (Ekonomim &amp; AA 7 Apr 2026)</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-04-07</t>
+          <t>ENRICHED 2026-10-20 · https://www.arabnews.com/node/2223976</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>BtcTurk</t>
+          <t>Saudi National Bank (SNB)</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>(position-only)</t>
+          <t>UNFILLED (position-only</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>CCO / MLRO (Head of Compliance / Uyum Muduru - not publicly named)</t>
+          <t>no public digital-assets/CCO lead identified)</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>Group CCO / digital assets lead</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr"/>
       <c r="G53" s="5" t="inlineStr"/>
       <c r="H53" s="5" t="inlineStr">
         <is>
-          <t>https://www.btcturk.com</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I53" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
+          <t>ENRICHED 2026-10-20 · https://news.google.com/rss/search?q=SNB+%22Saudi+National+Bank%22+chief+compliance+officer</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>Paribu</t>
+          <t>stc pay / STC Bank</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Yasin Oral</t>
+          <t>Mohammed Al-Fraih</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>CEO, Paribu (led CoinMENA acquisition Dec 2025 | quoted as CEO in deal coverage)</t>
+          <t>CEO of STC Bank (the licensed evolution of stc pay)</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -8639,268 +8639,268 @@
       <c r="G54" s="5" t="inlineStr"/>
       <c r="H54" s="5" t="inlineStr">
         <is>
-          <t>https://waya.media/paribu-acquires-majority-stake-in-coinmena-at-240m-valuation/</t>
+          <t>https://news.google.com/rss/search?q=%22stc+pay%22+CEO+appointed</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2025-12-07</t>
+          <t>ENRICHED 2026-10-20 · 2025-12-29</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>Paribu</t>
+          <t>stc pay / STC Bank</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Talal Tabba</t>
+          <t>UNFILLED (position-only</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Co-founder &amp; CEO, CoinMENA (Paribu group | owns MENA/Jordan expansion - CoinMENA entered Jordan under CBJ JoRegBox sandbox Sep 2026)</t>
+          <t>CCO not publicly named)</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>Chief Compliance Officer</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr"/>
       <c r="G55" s="5" t="inlineStr"/>
       <c r="H55" s="5" t="inlineStr">
         <is>
-          <t>https://www.coinmena.com/en/about (co-founder listed) + Khaleej Times (Tabba quoted as CoinMENA CEO) + fintekwins.com Jordan launch 28 Sep 2026</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-09-28</t>
+          <t>ENRICHED 2026-10-20 · https://news.google.com/rss/search?q=%22stc+pay%22+%22chief+compliance+officer%22</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>Paribu</t>
+          <t>Qatar Financial Centre Authority</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>Qatar</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>(position-only)</t>
+          <t>Mansoor Rashid Al-Khater</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>CCO / Head of Compliance (not publicly named | compliance org spans Paribu + CoinMENA CBB/VARA licences)</t>
+          <t>CEO of QFC (effective 11 Jan 2026, succeeding Yousuf Mohamed Al-Jaida)</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr"/>
       <c r="G56" s="5" t="inlineStr"/>
       <c r="H56" s="5" t="inlineStr">
         <is>
-          <t>https://www.paribu.com</t>
+          <t>https://www.thepeninsulaqatar.com/article/12/01/2026/qfc-welcomes-mansoor-rashid-al-khater-as-ceo</t>
         </is>
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
+          <t>ENRICHED 2026-10-20 · 2026-01-12</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>Binance TR</t>
+          <t>QFC Regulatory Authority</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>Qatar</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Mucahit Donmez</t>
+          <t>Michael Rayan</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>General Manager, Binance TR (active in role Sep 2026)</t>
+          <t>CEO of QFCRA (ran public consultation on Digital Assets Regulations)</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr"/>
       <c r="G57" s="5" t="inlineStr"/>
       <c r="H57" s="5" t="inlineStr">
         <is>
-          <t>https://www.teknotalk.com (TeknoTalk 8 Jun 2026: "Binance TR GM Mucahit Donmez" | prior Haberturk Sep 2023)</t>
+          <t>https://ffnews.com/newsarticle/regulatory/qfc-unveils-digital-assets-lab-powered-by-qcb-to-facilitate-open-innovation-in-qatar/</t>
         </is>
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-09-16</t>
+          <t>ENRICHED 2026-10-20 · 2023-10-31</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>OKX TR</t>
+          <t>Qatar Financial Centre Authority</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>Qatar</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Mehmet Camir</t>
+          <t>UNFILLED (position-only</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Chairman of the Board, OKX TR (Turkey JV with OKX)</t>
+          <t>Digital Assets Lab director not publicly named)</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>Digital Assets Lab / fintech innovation lead</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr"/>
       <c r="G58" s="5" t="inlineStr"/>
       <c r="H58" s="5" t="inlineStr">
         <is>
-          <t>https://www.halktv.com.tr (Halk TV 17 Mar 2026: "OKX TR YK Baskani Mehmet Camir")</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-03-17</t>
+          <t>ENRICHED 2026-10-20 · https://www.ledgerinsights.com/qatar-launches-digital-assets-lab/</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>HTTX</t>
+          <t>QNB Group</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>Qatar</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>(position-only)</t>
+          <t>UNFILLED (position-only</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>CEO / General Manager (Turkish crypto platform | no 2025-2026 named executive found in news sources - honest gap)</t>
+          <t>digital-asset evaluation lead not publicly named</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>low</t>
+          <t xml:space="preserve"> MoUs signed at Web Summit Qatar 2025)</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr"/>
       <c r="G59" s="5" t="inlineStr"/>
       <c r="H59" s="5" t="inlineStr">
         <is>
-          <t>https://www.cnbc-e.com (crypto sector coverage | HTTX leadership not covered)</t>
+          <t>Digital assets evaluation lead</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
+          <t>ENRICHED 2026-10-20 · low</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>Garanti BBVA Kripto</t>
+          <t>Qatar Central Bank</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>Qatar</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Onur Guven</t>
+          <t>Sheikh Bandar bin Mohammed bin Saoud Al-Thani</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>General Manager, Garanti BBVA Kripto (appointed Jan 2025 | platform still led by him through OTC launch Jul 2026)</t>
+          <t>Governor (since Nov 2021</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t xml:space="preserve"> patron of QFC Digital Assets Lab under QCB Fintech Strategy)</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr"/>
       <c r="G60" s="5" t="inlineStr"/>
       <c r="H60" s="5" t="inlineStr">
         <is>
-          <t>https://www.haberturk.com (Haberturk 10 Jan 2025 | AA 9 Jul 2026 OTC launch)</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-07-09</t>
+          <t>ENRICHED 2026-10-20 · https://www.qcb.gov.qa/en/Pages/Governor.aspx</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>Papara / inPay</t>
+          <t>CMA Kuwait</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>Kuwait</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Ahmet Faruk Karsli</t>
+          <t>Emad Ahmed Tifouni</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Founder &amp; former owner, Papara (arrested Jul 2026 in illegal-betting probe | assets liquidated - Papara sold out of TMSF custody to Emlak Katilim Bankasi Apr 2026)</t>
+          <t>Chairman of CMA Board of Commissioners &amp; Managing Director (Fourth Board, since April 2025)</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -8912,163 +8912,163 @@
       <c r="G61" s="5" t="inlineStr"/>
       <c r="H61" s="5" t="inlineStr">
         <is>
-          <t>https://www.evrensel.net (Evrensel 10 Jul 2026 re-arrest | T24/Forbes Turkiye 17 Apr 2026 sale to Emlak Katilim)</t>
+          <t>https://www.cma.gov.kw/en/web/cma/fourth-board</t>
         </is>
       </c>
       <c r="I61" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-07-10</t>
+          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>Papara / inPay</t>
+          <t>CMA Kuwait</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>Kuwait</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>(position-only)</t>
+          <t>UNFILLED (position-only</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>CEO under new owner (Emlak Katilim Bankasi control) + CCO - not publicly named</t>
+          <t>CMA runs absolute VA ban regime and AML coordination incl. Nazaha MoU 2026)</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>VA-framework / AML consultation owner</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr"/>
       <c r="G62" s="5" t="inlineStr"/>
       <c r="H62" s="5" t="inlineStr">
         <is>
-          <t>https://www.cnbc-e.com (16 Apr 2026)</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-04-16</t>
+          <t>ENRICHED 2026-10-20 · https://news.google.com/rss/search?q=Nazaha+FIU+deepen+alliance</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>FRA (Financial Regulatory Authority)</t>
+          <t>Boubyan Bank</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>Kuwait</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Islam Azzam</t>
+          <t>Adel Al-Majed</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Chairman, FRA (appointed Mar 2026 | elected IOSCO Vice Chair Apr 2026 | oversees Law 162/2023 virtual-assets regime)</t>
+          <t>Group Vice Chairman &amp; CEO (confirmed in IMF/WB Kuwait banks coverage Oct 2026</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>high</t>
+          <t xml:space="preserve"> a May 2026 Kuwait Times headline references a different surname 'Al-Tuwaijri' as CEO - verify)</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr"/>
       <c r="G63" s="5" t="inlineStr"/>
       <c r="H63" s="5" t="inlineStr">
         <is>
-          <t>https://enterpriseam.com/egypts-financial-regulatory-authority-appoints-islam-azzam-as-new-head/</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I63" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-03-10</t>
+          <t>ENRICHED 2026-10-20 · https://timeskuwait.com/kuwaiti-banks-showcase-financial-strength-at-imf-world-bank-meetings/</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>FRA (Financial Regulatory Authority)</t>
+          <t>Boubyan Bank</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>Kuwait</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Mohamed Farid</t>
+          <t>UNFILLED (position-only</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Former FRA Chairman (through Jan 2026 | superseded by Azzam)</t>
+          <t>digital-assets/compliance head not publicly named)</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>Head of compliance / digital assets</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr"/>
       <c r="G64" s="5" t="inlineStr"/>
       <c r="H64" s="5" t="inlineStr">
         <is>
-          <t>https://www.dailynewsegypt.com (Feb 2025 "Farid emphasises strengthening non-bank financial sector resilience")</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-01-31</t>
+          <t>ENRICHED 2026-10-20 · https://news.google.com/rss/search?q=Boubyan+Bank+CEO+Kuwait</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>FRA (Financial Regulatory Authority)</t>
+          <t>Financial Services Authority Oman (successor to CMA Oman, est. 2024)</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>Oman</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>(position-only)</t>
+          <t>Dr. Khamis Saif Al Jabri</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Head of AML compliance / virtual-assets supervision under Law 162/2023 (not publicly named)</t>
+          <t>Minister of Economy - Chairman of FSA Board of Directors</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr"/>
       <c r="G65" s="5" t="inlineStr"/>
       <c r="H65" s="5" t="inlineStr">
         <is>
-          <t>https://www.fra.org.eg</t>
+          <t>https://www.fsa.gov.om/Home/AboutCMA/BoardofDirectors</t>
         </is>
       </c>
       <c r="I65" s="5" t="inlineStr">
@@ -9080,178 +9080,178 @@
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>Egypt FRA-licensed VASP cohort</t>
+          <t>Sohar International</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>Oman</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>(position-only)</t>
+          <t>Abdulwahid Almurshidi</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>First licensed virtual-asset companies (executive-regulations licensing in progress through 2026 | no company names confirmed in 2025-2026 FRA announcements accessible to this research - honest gap)</t>
+          <t>Chief Executive Officer (named Feb 2025)</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr"/>
       <c r="G66" s="5" t="inlineStr"/>
       <c r="H66" s="5" t="inlineStr">
         <is>
-          <t>https://www.iflr.com (IFLR Egyptian capital market developments, Oct 2025)</t>
+          <t>https://news.google.com/rss/search?q=Sohar+International+CEO+2025</t>
         </is>
       </c>
       <c r="I66" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
+          <t>ENRICHED 2026-10-20 · 2025-02-26</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>Egypt FIU (Unit for Combating Money Laundering and Financing Terrorism, EEFFU)</t>
+          <t>NBO National Bank of Oman</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>Oman</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Ahmed Khalil (al-Mustashar Ahmed Khalil)</t>
+          <t>UNFILLED (position-only</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>Head of Egypt's AML/CFT Unit (quoted in role Jun-Sep 2026 | MOU with China FIU Aug 2026)</t>
+          <t>CEO and digital-assets lead not verifiable in this pass)</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>CEO / digital assets lead</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr"/>
       <c r="G67" s="5" t="inlineStr"/>
       <c r="H67" s="5" t="inlineStr">
         <is>
-          <t>https://www.ahram.org.eg (Akhbar Al-Youm 7 Jul 2026 | SIE 3 Oct 2026 FRA-FIU joint event)</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I67" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-09-07</t>
+          <t>ENRICHED 2026-10-20 · https://news.google.com/rss/search?q=National+Bank+of+Oman+digital</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>CIB Egypt / Yomo</t>
+          <t>MENAFATF (secretariat seated Manama, Bahrain)</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>Bahrain (MENA body)</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Rashwan Hamady</t>
+          <t>Suliman Aljabrin</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>CEO &amp; Managing Director, Yomo (CIB's digital bank - closest CIB digital-assets banking executive)</t>
+          <t>Executive Secretary (since 1 Jan 2021</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t xml:space="preserve"> ex-SAMA Banking Policy Director</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr"/>
       <c r="G68" s="5" t="inlineStr"/>
       <c r="H68" s="5" t="inlineStr">
         <is>
-          <t>https://www.fin-tech-gate.com (Fintech Gate / FRA-affiliated portal 20 Aug 2026)</t>
+          <t xml:space="preserve"> verify current incumbency)</t>
         </is>
       </c>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-08-20</t>
+          <t>ENRICHED 2026-10-20 · medium</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>CIB Egypt</t>
+          <t>IFZA (Dubai freezone onboarding)</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Kamran Bader</t>
+          <t>Philipp Conrads (CEO IFZA Dubai) / Jochen Knecht (CEO IFZA Global)</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>Chief Data, Analytics &amp; AI Officer, CIB Egypt</t>
+          <t>Freezone compliance-services leads</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr"/>
       <c r="G69" s="5" t="inlineStr"/>
       <c r="H69" s="5" t="inlineStr">
         <is>
-          <t>https://hrtoday.in (Jun 2026)</t>
+          <t>https://ifza.com/en/leadership/</t>
         </is>
       </c>
       <c r="I69" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-06-04</t>
+          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>Jordan Securities Commission</t>
+          <t>RAKEZ (Ras Al Khaimah Economic Zone)</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>JO</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Emad Muhammad Abuhaltam</t>
+          <t>Ramy Jallad</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>Chairman of the Board of Commissioners &amp; CEO (JSC runs virtual-asset licensing | "Preliminary Approval to Practice Virtual Assets Activities" form live on site)</t>
+          <t>Group CEO of RAKEZ</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -9263,34 +9263,34 @@
       <c r="G70" s="5" t="inlineStr"/>
       <c r="H70" s="5" t="inlineStr">
         <is>
-          <t>https://www.jsc.gov.jo/page/en/chairman_and_board_of_commissioners (official site, last update 19/10/2026)</t>
+          <t>https://usa.chinadaily.com.cn/a/202609/08/WS6a9fd15de4b06d4aa055cf48.html</t>
         </is>
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-19</t>
+          <t>ENRICHED 2026-10-20 · 2026-09-08</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>Jordan Securities Commission</t>
+          <t>DMCC (incl. 500+ crypto member community)</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>JO</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Elias Ayoub Zoreikat</t>
+          <t>Ahmed Bin Sulayem</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>Deputy Chairman, JSC Board of Commissioners</t>
+          <t>Executive Chairman &amp; CEO (Deputy CEO/COO: Feryal Ahmadi)</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -9302,34 +9302,34 @@
       <c r="G71" s="5" t="inlineStr"/>
       <c r="H71" s="5" t="inlineStr">
         <is>
-          <t>https://www.jsc.gov.jo/page/en/chairman_and_board_of_commissioners</t>
+          <t>https://www.dmcc.ae/about-us</t>
         </is>
       </c>
       <c r="I71" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-19</t>
+          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>Jordan Securities Commission</t>
+          <t>Deloitte Middle East</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>JO</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Razan Samih Al-Shafei</t>
+          <t>Simon Cuerden</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>Commissioner, JSC Board of Commissioners</t>
+          <t>Leader, Forensic &amp; Financial Crime practice (Middle East)</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -9341,34 +9341,34 @@
       <c r="G72" s="5" t="inlineStr"/>
       <c r="H72" s="5" t="inlineStr">
         <is>
-          <t>https://www.jsc.gov.jo/page/en/chairman_and_board_of_commissioners</t>
+          <t>https://www.consultancy-me.com/news/8737/simon-cuerden-new-leader-of-deloittes-forensic-financial-crime-business</t>
         </is>
       </c>
       <c r="I72" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-19</t>
+          <t>ENRICHED 2026-10-20 · 2025-01-10</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>Jordan - first regulated VASP</t>
+          <t>FTI Consulting (MENA financial-crime practice)</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>JO</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>(position-only)</t>
+          <t>Abi-gail Marshman</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>CoinMENA (Paribu group) - first digital-asset trading platform admitted to Central Bank of Jordan JoRegBox regulatory sandbox (Sep 2026, live with CliQ JOD rails) |position-only row (first in-market entity, per Turkish/MENA trade press)</t>
+          <t>Head of Financial Crime for MENA (2022 appointment - verify current)</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -9380,151 +9380,151 @@
       <c r="G73" s="5" t="inlineStr"/>
       <c r="H73" s="5" t="inlineStr">
         <is>
-          <t>https://fintekwins.com/paribu-coinmena-ile-urdun-pazarina-girdi/</t>
+          <t>https://www.consultancy-me.com/news/7321/abi-gail-marshman-joins-fti-as-head-of-financial-crime-for-mena</t>
         </is>
       </c>
       <c r="I73" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-09-28</t>
+          <t>ENRICHED 2026-10-20 · 2022-09-06</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>Lebanon FIU (Special Investigation Commission on Money Laundering / SCLC)</t>
+          <t>KPMG Middle East</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>(position-only)</t>
+          <t>UNFILLED (position-only</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Chairperson of SCLC (judicially chaired body | current chair not confirmable from accessible 2025-2026 sources - honest gap | commission active, demanded bank data for 11 persons Sep 2026)</t>
+          <t>no named regional financial-crime practice head found)</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>Regional AML/financial-crime practice leader</t>
         </is>
       </c>
       <c r="F74" s="5" t="inlineStr"/>
       <c r="G74" s="5" t="inlineStr"/>
       <c r="H74" s="5" t="inlineStr">
         <is>
-          <t>https://www.libnanews.com (24 Sep 2026)</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I74" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-09-24</t>
+          <t>ENRICHED 2026-10-20 · https://news.google.com/rss/search?q=KPMG+Middle+East+%22financial+crime%22</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>Banque du Liban</t>
+          <t>EY Middle East</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Karim Souaid</t>
+          <t>UNFILLED (position-only</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>Governor of Banque du Liban (appointed Mar 2025 | payments/digital-currency reform agenda | crypto framework owner at recentral bank)</t>
+          <t>EY Crypto Financial Crime CoE is US-listed)</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>Regional AML/financial-crime practice leader</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr"/>
       <c r="G75" s="5" t="inlineStr"/>
       <c r="H75" s="5" t="inlineStr">
         <is>
-          <t>https://www.reuters.com (Reuters 27 Mar 2025 "Lebanon appoints asset manager Karim Souaid as new central bank governor")</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I75" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2025-03-27</t>
+          <t>ENRICHED 2026-10-20 · https://www.ey.com/en_us/services/consulting/financial-crime-crypto-center-of-excellence</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>Banque du Liban</t>
+          <t>PwC Middle East</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>(position-only)</t>
+          <t>UNFILLED (position-only</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>Head of payments / digital-assets unit (reform-era unit | individual not publicly named)</t>
+          <t>FCS/managed-services financial-crime lead not named)</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>Regional AML/financial-crime practice leader</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr"/>
       <c r="G76" s="5" t="inlineStr"/>
       <c r="H76" s="5" t="inlineStr">
         <is>
-          <t>https://bdl.com.lb</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I76" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
+          <t>ENRICHED 2026-10-20 · https://www.pwc.com/m1/en/services/consulting/financial-crime-management.html</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>AMMC (Morocco capital-markets regulator)</t>
+          <t>SPK (Sermaye Piyasasi Kurulu / Capital Markets Board)</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Tarik Senhaji</t>
+          <t>Mahmut Sutcu</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>Secretary General / de facto head of AMMC (presents 2026 action priorities and speaks as AMMC principal in 2026 press | digital-asset mandate under law 43-21 framework pending implementing texts)</t>
+          <t>Kurul Chairman (appointed 9 May 2026 | removed from office 19-20 Oct 2026, successor not yet named at time of research)</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -9536,24 +9536,24 @@
       <c r="G77" s="5" t="inlineStr"/>
       <c r="H77" s="5" t="inlineStr">
         <is>
-          <t>https://le360.ma (Le360 23 Jun 2026 "l'AMMC deroule sa strategie" | Le Desk 28 Jan 2026 "Senhaji devoile les priorites d'actions de l'AMMC pour 2026")</t>
+          <t>https://www.dunya.com (Dunya Gazetesi: "SPK Baskani Mahmut Sutcu ve KGK Baskani Ibrahim Omer Gonul gorevden alindi", 20 Oct 2026 | original appointment: A Haber 9 May 2026, tr.wikipedia.org/wiki/Sermaye_Piyasas%C4%B1_Kurumu)</t>
         </is>
       </c>
       <c r="I77" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-09-30</t>
+          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>AMMC</t>
+          <t>SPK (Sermaye Piyasasi Kurulu)</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
@@ -9563,7 +9563,7 @@
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>Digital-assets / innovation division lead under law 43-21 (crypto bill draft published Nov 2025 | division head not publicly named)</t>
+          <t>Head of digital-assets / crypto licensing division (SPK oversees VASP licensing under Law 7518 | division head not publicly named)</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -9575,34 +9575,34 @@
       <c r="G78" s="5" t="inlineStr"/>
       <c r="H78" s="5" t="inlineStr">
         <is>
-          <t>https://medias24.com (3 Nov 2025 avant-projet de loi crypto)</t>
+          <t>https://spk.gov.tr/hakkimizda/kurul-baskani</t>
         </is>
       </c>
       <c r="I78" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2025-11-03</t>
+          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>Bank Al-Maghrib</t>
+          <t>MASAK (Financial Crimes Investigation Board)</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Abdellatif Jouahri</t>
+          <t>Hasan Kaymak</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>Wali (Governor), Bank Al-Maghrib (crypto-activities ban stance owner | annual report presented to King Jul 2026 | active through Sep 2026 MPC)</t>
+          <t>President of MASAK (appointed Feb 2024 | publicly active as MASAK head Oct 2026)</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -9614,24 +9614,24 @@
       <c r="G79" s="5" t="inlineStr"/>
       <c r="H79" s="5" t="inlineStr">
         <is>
-          <t>https://medias24.com (21 Jul 2026 Jouahri presents BAM annual report to Mohammed VI | SNRT 22 Sep 2026)</t>
+          <t>https://www.aa.com.tr (Anadolu/AHaber 23 Feb 2024 | Anka Haber 14 Oct 2026 "MASAK Baskani Kaymak")</t>
         </is>
       </c>
       <c r="I79" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-09-22</t>
+          <t>ENRICHED 2026-10-20 · 2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>Bank Al-Maghrib</t>
+          <t>MASAK (Financial Crimes Investigation Board)</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
@@ -9641,7 +9641,7 @@
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>Digital payments / asset tokenisation programme owner (not publicly named)</t>
+          <t>Uyum / compliance programme lead (AML compliance supervision directorate | individual not publicly named)</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -9653,7 +9653,7 @@
       <c r="G80" s="5" t="inlineStr"/>
       <c r="H80" s="5" t="inlineStr">
         <is>
-          <t>https://bkam.ma</t>
+          <t>https://www.masak.gov.tr</t>
         </is>
       </c>
       <c r="I80" s="5" t="inlineStr">
@@ -9665,139 +9665,139 @@
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>Central Bank of Iraq (CBQ/CBI)</t>
+          <t>BtcTurk</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>IQ</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Nizar (Hussein/Nasir) - full transliteration varies across sources</t>
+          <t>Tevfik Kinik</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>Governor of the Central Bank of Iraq (appointed Jun 2026, replacing Ali Al-Alaq | oversaw Oct 2026 dinar re-peg to 1,500 IQD/USD)</t>
+          <t>CEO of BtcTurk Group Companies (appointed Jan 2026)</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F81" s="5" t="inlineStr"/>
       <c r="G81" s="5" t="inlineStr"/>
       <c r="H81" s="5" t="inlineStr">
         <is>
-          <t>https://enterpriseam.com (24 Jun 2026 "Iraq appoints Nizar Hussein as new central bank governor") + en.wikipedia.org/wiki/Central_Bank_of_Iraq ("Nizar Nasir" infobox, Baghdad Today citation)</t>
+          <t>https://www.aa.com.tr (Anadolu Ajansi &amp; DHA 6 Jan 2026 "BtcTurk'te ust duzey atama" | Fortune Turkey)</t>
         </is>
       </c>
       <c r="I81" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-06-24</t>
+          <t>ENRICHED 2026-10-20 · 2026-01-06</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>Central Bank of Iraq</t>
+          <t>BtcTurk</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>IQ</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>(position-only)</t>
+          <t>Fatih Otluoglu</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>Deputy Governor for Payments / FX-corridor oversight (dinar-dollar corridor owner | individual not confirmable from accessible sources - corpus-only account, low effort per brief)</t>
+          <t>CEO of BtcTurk Hisse (brokerage arm)</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr"/>
       <c r="G82" s="5" t="inlineStr"/>
       <c r="H82" s="5" t="inlineStr">
         <is>
-          <t>https://cbi.iq</t>
+          <t>https://www.ekonomim.com (Ekonomim &amp; AA 7 Apr 2026)</t>
         </is>
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
+          <t>ENRICHED 2026-10-20 · 2026-04-07</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>VARA (Dubai)</t>
+          <t>BtcTurk</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>UAE</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Helal Saeed Almarri</t>
+          <t>(position-only)</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>Chairman of Executive Board</t>
+          <t>CCO / MLRO (Head of Compliance / Uyum Muduru - not publicly named)</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="F83" s="5" t="inlineStr"/>
       <c r="G83" s="5" t="inlineStr"/>
       <c r="H83" s="5" t="inlineStr">
         <is>
-          <t>https://www.vara.ae/en/about-vara/</t>
+          <t>https://www.btcturk.com</t>
         </is>
       </c>
       <c r="I83" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-20 rescued (subagent leg failed to compile)</t>
+          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>CoinMENA</t>
+          <t>Paribu</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>Bahrain</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Talal Tabbaa</t>
+          <t>Yasin Oral</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>Co-Founder</t>
+          <t>CEO, Paribu (led CoinMENA acquisition Dec 2025 | quoted as CEO in deal coverage)</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -9809,112 +9809,112 @@
       <c r="G84" s="5" t="inlineStr"/>
       <c r="H84" s="5" t="inlineStr">
         <is>
-          <t>https://www.coinmena.com/en/about-us</t>
+          <t>https://waya.media/paribu-acquires-majority-stake-in-coinmena-at-240m-valuation/</t>
         </is>
       </c>
       <c r="I84" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-20 rescued</t>
+          <t>ENRICHED 2026-10-20 · 2025-12-07</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>CoinMENA</t>
+          <t>Paribu</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>Bahrain</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Dina Sam'an</t>
+          <t>Talal Tabba</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>Co-Founder</t>
+          <t>Co-founder &amp; CEO, CoinMENA (Paribu group | owns MENA/Jordan expansion - CoinMENA entered Jordan under CBJ JoRegBox sandbox Sep 2026)</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="F85" s="5" t="inlineStr"/>
       <c r="G85" s="5" t="inlineStr"/>
       <c r="H85" s="5" t="inlineStr">
         <is>
-          <t>https://www.coinmena.com/en/about-us</t>
+          <t>https://www.coinmena.com/en/about (co-founder listed) + Khaleej Times (Tabba quoted as CoinMENA CEO) + fintekwins.com Jordan launch 28 Sep 2026</t>
         </is>
       </c>
       <c r="I85" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-20 rescued</t>
+          <t>ENRICHED 2026-10-20 · 2026-09-28</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>CoinMENA</t>
+          <t>Paribu</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Bahrain</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Yazan Barghuthi</t>
+          <t>(position-only)</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>Co-Founder</t>
+          <t>CCO / Head of Compliance (not publicly named | compliance org spans Paribu + CoinMENA CBB/VARA licences)</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="F86" s="5" t="inlineStr"/>
       <c r="G86" s="5" t="inlineStr"/>
       <c r="H86" s="5" t="inlineStr">
         <is>
-          <t>https://www.coinmena.com/en/about-us</t>
+          <t>https://www.paribu.com</t>
         </is>
       </c>
       <c r="I86" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-20 rescued</t>
+          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>DMCC Crypto Centre</t>
+          <t>Binance TR</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>UAE</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>H.E. Mansour Mohamed AlMulla</t>
+          <t>Mucahit Donmez</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>Chairman (also Deputy Group CEO, ADQ)</t>
+          <t>General Manager, Binance TR (active in role Sep 2026)</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -9926,49 +9926,1219 @@
       <c r="G87" s="5" t="inlineStr"/>
       <c r="H87" s="5" t="inlineStr">
         <is>
-          <t>https://dmcc.ae/latest-news</t>
+          <t>https://www.teknotalk.com (TeknoTalk 8 Jun 2026: "Binance TR GM Mucahit Donmez" | prior Haberturk Sep 2023)</t>
         </is>
       </c>
       <c r="I87" s="5" t="inlineStr">
         <is>
-          <t>ENRICHED 2026-10-20 · 2026-10-20 rescued</t>
+          <t>ENRICHED 2026-10-20 · 2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>Zand (UAE digital bank)</t>
+          <t>OKX TR</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>UAE</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>(position-only)</t>
+          <t>Mehmet Camir</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>AI-powered bank partnered with CoinMENA fiat-crypto integration = prospect discovery</t>
+          <t>Chairman of the Board, OKX TR (Turkey JV with OKX)</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr"/>
       <c r="G88" s="5" t="inlineStr"/>
       <c r="H88" s="5" t="inlineStr">
         <is>
+          <t>https://www.halktv.com.tr (Halk TV 17 Mar 2026: "OKX TR YK Baskani Mehmet Camir")</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-03-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>HTTX</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>(position-only)</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>CEO / General Manager (Turkish crypto platform | no 2025-2026 named executive found in news sources - honest gap)</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F89" s="5" t="inlineStr"/>
+      <c r="G89" s="5" t="inlineStr"/>
+      <c r="H89" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cnbc-e.com (crypto sector coverage | HTTX leadership not covered)</t>
+        </is>
+      </c>
+      <c r="I89" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>Garanti BBVA Kripto</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Onur Guven</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>General Manager, Garanti BBVA Kripto (appointed Jan 2025 | platform still led by him through OTC launch Jul 2026)</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr"/>
+      <c r="G90" s="5" t="inlineStr"/>
+      <c r="H90" s="5" t="inlineStr">
+        <is>
+          <t>https://www.haberturk.com (Haberturk 10 Jan 2025 | AA 9 Jul 2026 OTC launch)</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-07-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>Papara / inPay</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>Ahmet Faruk Karsli</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>Founder &amp; former owner, Papara (arrested Jul 2026 in illegal-betting probe | assets liquidated - Papara sold out of TMSF custody to Emlak Katilim Bankasi Apr 2026)</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F91" s="5" t="inlineStr"/>
+      <c r="G91" s="5" t="inlineStr"/>
+      <c r="H91" s="5" t="inlineStr">
+        <is>
+          <t>https://www.evrensel.net (Evrensel 10 Jul 2026 re-arrest | T24/Forbes Turkiye 17 Apr 2026 sale to Emlak Katilim)</t>
+        </is>
+      </c>
+      <c r="I91" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>Papara / inPay</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>(position-only)</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>CEO under new owner (Emlak Katilim Bankasi control) + CCO - not publicly named</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F92" s="5" t="inlineStr"/>
+      <c r="G92" s="5" t="inlineStr"/>
+      <c r="H92" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cnbc-e.com (16 Apr 2026)</t>
+        </is>
+      </c>
+      <c r="I92" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-04-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>FRA (Financial Regulatory Authority)</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>Islam Azzam</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>Chairman, FRA (appointed Mar 2026 | elected IOSCO Vice Chair Apr 2026 | oversees Law 162/2023 virtual-assets regime)</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F93" s="5" t="inlineStr"/>
+      <c r="G93" s="5" t="inlineStr"/>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t>https://enterpriseam.com/egypts-financial-regulatory-authority-appoints-islam-azzam-as-new-head/</t>
+        </is>
+      </c>
+      <c r="I93" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-03-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
+        <is>
+          <t>FRA (Financial Regulatory Authority)</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Mohamed Farid</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>Former FRA Chairman (through Jan 2026 | superseded by Azzam)</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="inlineStr"/>
+      <c r="G94" s="5" t="inlineStr"/>
+      <c r="H94" s="5" t="inlineStr">
+        <is>
+          <t>https://www.dailynewsegypt.com (Feb 2025 "Farid emphasises strengthening non-bank financial sector resilience")</t>
+        </is>
+      </c>
+      <c r="I94" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-01-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t>FRA (Financial Regulatory Authority)</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>(position-only)</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>Head of AML compliance / virtual-assets supervision under Law 162/2023 (not publicly named)</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F95" s="5" t="inlineStr"/>
+      <c r="G95" s="5" t="inlineStr"/>
+      <c r="H95" s="5" t="inlineStr">
+        <is>
+          <t>https://www.fra.org.eg</t>
+        </is>
+      </c>
+      <c r="I95" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>Egypt FRA-licensed VASP cohort</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>(position-only)</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>First licensed virtual-asset companies (executive-regulations licensing in progress through 2026 | no company names confirmed in 2025-2026 FRA announcements accessible to this research - honest gap)</t>
+        </is>
+      </c>
+      <c r="E96" s="5" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F96" s="5" t="inlineStr"/>
+      <c r="G96" s="5" t="inlineStr"/>
+      <c r="H96" s="5" t="inlineStr">
+        <is>
+          <t>https://www.iflr.com (IFLR Egyptian capital market developments, Oct 2025)</t>
+        </is>
+      </c>
+      <c r="I96" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>Egypt FIU (Unit for Combating Money Laundering and Financing Terrorism, EEFFU)</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>Ahmed Khalil (al-Mustashar Ahmed Khalil)</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>Head of Egypt's AML/CFT Unit (quoted in role Jun-Sep 2026 | MOU with China FIU Aug 2026)</t>
+        </is>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F97" s="5" t="inlineStr"/>
+      <c r="G97" s="5" t="inlineStr"/>
+      <c r="H97" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ahram.org.eg (Akhbar Al-Youm 7 Jul 2026 | SIE 3 Oct 2026 FRA-FIU joint event)</t>
+        </is>
+      </c>
+      <c r="I97" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="inlineStr">
+        <is>
+          <t>CIB Egypt / Yomo</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>Rashwan Hamady</t>
+        </is>
+      </c>
+      <c r="D98" s="5" t="inlineStr">
+        <is>
+          <t>CEO &amp; Managing Director, Yomo (CIB's digital bank - closest CIB digital-assets banking executive)</t>
+        </is>
+      </c>
+      <c r="E98" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F98" s="5" t="inlineStr"/>
+      <c r="G98" s="5" t="inlineStr"/>
+      <c r="H98" s="5" t="inlineStr">
+        <is>
+          <t>https://www.fin-tech-gate.com (Fintech Gate / FRA-affiliated portal 20 Aug 2026)</t>
+        </is>
+      </c>
+      <c r="I98" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-08-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>CIB Egypt</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>Kamran Bader</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>Chief Data, Analytics &amp; AI Officer, CIB Egypt</t>
+        </is>
+      </c>
+      <c r="E99" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F99" s="5" t="inlineStr"/>
+      <c r="G99" s="5" t="inlineStr"/>
+      <c r="H99" s="5" t="inlineStr">
+        <is>
+          <t>https://hrtoday.in (Jun 2026)</t>
+        </is>
+      </c>
+      <c r="I99" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="5" t="inlineStr">
+        <is>
+          <t>Jordan Securities Commission</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Emad Muhammad Abuhaltam</t>
+        </is>
+      </c>
+      <c r="D100" s="5" t="inlineStr">
+        <is>
+          <t>Chairman of the Board of Commissioners &amp; CEO (JSC runs virtual-asset licensing | "Preliminary Approval to Practice Virtual Assets Activities" form live on site)</t>
+        </is>
+      </c>
+      <c r="E100" s="5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F100" s="5" t="inlineStr"/>
+      <c r="G100" s="5" t="inlineStr"/>
+      <c r="H100" s="5" t="inlineStr">
+        <is>
+          <t>https://www.jsc.gov.jo/page/en/chairman_and_board_of_commissioners (official site, last update 19/10/2026)</t>
+        </is>
+      </c>
+      <c r="I100" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>Jordan Securities Commission</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>Elias Ayoub Zoreikat</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>Deputy Chairman, JSC Board of Commissioners</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F101" s="5" t="inlineStr"/>
+      <c r="G101" s="5" t="inlineStr"/>
+      <c r="H101" s="5" t="inlineStr">
+        <is>
+          <t>https://www.jsc.gov.jo/page/en/chairman_and_board_of_commissioners</t>
+        </is>
+      </c>
+      <c r="I101" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="inlineStr">
+        <is>
+          <t>Jordan Securities Commission</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>Razan Samih Al-Shafei</t>
+        </is>
+      </c>
+      <c r="D102" s="5" t="inlineStr">
+        <is>
+          <t>Commissioner, JSC Board of Commissioners</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F102" s="5" t="inlineStr"/>
+      <c r="G102" s="5" t="inlineStr"/>
+      <c r="H102" s="5" t="inlineStr">
+        <is>
+          <t>https://www.jsc.gov.jo/page/en/chairman_and_board_of_commissioners</t>
+        </is>
+      </c>
+      <c r="I102" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>Jordan - first regulated VASP</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>(position-only)</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>CoinMENA (Paribu group) - first digital-asset trading platform admitted to Central Bank of Jordan JoRegBox regulatory sandbox (Sep 2026, live with CliQ JOD rails) |position-only row (first in-market entity, per Turkish/MENA trade press)</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F103" s="5" t="inlineStr"/>
+      <c r="G103" s="5" t="inlineStr"/>
+      <c r="H103" s="5" t="inlineStr">
+        <is>
+          <t>https://fintekwins.com/paribu-coinmena-ile-urdun-pazarina-girdi/</t>
+        </is>
+      </c>
+      <c r="I103" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="5" t="inlineStr">
+        <is>
+          <t>Lebanon FIU (Special Investigation Commission on Money Laundering / SCLC)</t>
+        </is>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>(position-only)</t>
+        </is>
+      </c>
+      <c r="D104" s="5" t="inlineStr">
+        <is>
+          <t>Chairperson of SCLC (judicially chaired body | current chair not confirmable from accessible 2025-2026 sources - honest gap | commission active, demanded bank data for 11 persons Sep 2026)</t>
+        </is>
+      </c>
+      <c r="E104" s="5" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F104" s="5" t="inlineStr"/>
+      <c r="G104" s="5" t="inlineStr"/>
+      <c r="H104" s="5" t="inlineStr">
+        <is>
+          <t>https://www.libnanews.com (24 Sep 2026)</t>
+        </is>
+      </c>
+      <c r="I104" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="inlineStr">
+        <is>
+          <t>Banque du Liban</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>Karim Souaid</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>Governor of Banque du Liban (appointed Mar 2025 | payments/digital-currency reform agenda | crypto framework owner at recentral bank)</t>
+        </is>
+      </c>
+      <c r="E105" s="5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F105" s="5" t="inlineStr"/>
+      <c r="G105" s="5" t="inlineStr"/>
+      <c r="H105" s="5" t="inlineStr">
+        <is>
+          <t>https://www.reuters.com (Reuters 27 Mar 2025 "Lebanon appoints asset manager Karim Souaid as new central bank governor")</t>
+        </is>
+      </c>
+      <c r="I105" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2025-03-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr">
+        <is>
+          <t>Banque du Liban</t>
+        </is>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>(position-only)</t>
+        </is>
+      </c>
+      <c r="D106" s="5" t="inlineStr">
+        <is>
+          <t>Head of payments / digital-assets unit (reform-era unit | individual not publicly named)</t>
+        </is>
+      </c>
+      <c r="E106" s="5" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F106" s="5" t="inlineStr"/>
+      <c r="G106" s="5" t="inlineStr"/>
+      <c r="H106" s="5" t="inlineStr">
+        <is>
+          <t>https://bdl.com.lb</t>
+        </is>
+      </c>
+      <c r="I106" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="inlineStr">
+        <is>
+          <t>AMMC (Morocco capital-markets regulator)</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>Tarik Senhaji</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>Secretary General / de facto head of AMMC (presents 2026 action priorities and speaks as AMMC principal in 2026 press | digital-asset mandate under law 43-21 framework pending implementing texts)</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F107" s="5" t="inlineStr"/>
+      <c r="G107" s="5" t="inlineStr"/>
+      <c r="H107" s="5" t="inlineStr">
+        <is>
+          <t>https://le360.ma (Le360 23 Jun 2026 "l'AMMC deroule sa strategie" | Le Desk 28 Jan 2026 "Senhaji devoile les priorites d'actions de l'AMMC pour 2026")</t>
+        </is>
+      </c>
+      <c r="I107" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="5" t="inlineStr">
+        <is>
+          <t>AMMC</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>(position-only)</t>
+        </is>
+      </c>
+      <c r="D108" s="5" t="inlineStr">
+        <is>
+          <t>Digital-assets / innovation division lead under law 43-21 (crypto bill draft published Nov 2025 | division head not publicly named)</t>
+        </is>
+      </c>
+      <c r="E108" s="5" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F108" s="5" t="inlineStr"/>
+      <c r="G108" s="5" t="inlineStr"/>
+      <c r="H108" s="5" t="inlineStr">
+        <is>
+          <t>https://medias24.com (3 Nov 2025 avant-projet de loi crypto)</t>
+        </is>
+      </c>
+      <c r="I108" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2025-11-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="5" t="inlineStr">
+        <is>
+          <t>Bank Al-Maghrib</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>Abdellatif Jouahri</t>
+        </is>
+      </c>
+      <c r="D109" s="5" t="inlineStr">
+        <is>
+          <t>Wali (Governor), Bank Al-Maghrib (crypto-activities ban stance owner | annual report presented to King Jul 2026 | active through Sep 2026 MPC)</t>
+        </is>
+      </c>
+      <c r="E109" s="5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F109" s="5" t="inlineStr"/>
+      <c r="G109" s="5" t="inlineStr"/>
+      <c r="H109" s="5" t="inlineStr">
+        <is>
+          <t>https://medias24.com (21 Jul 2026 Jouahri presents BAM annual report to Mohammed VI | SNRT 22 Sep 2026)</t>
+        </is>
+      </c>
+      <c r="I109" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-09-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="5" t="inlineStr">
+        <is>
+          <t>Bank Al-Maghrib</t>
+        </is>
+      </c>
+      <c r="B110" s="5" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>(position-only)</t>
+        </is>
+      </c>
+      <c r="D110" s="5" t="inlineStr">
+        <is>
+          <t>Digital payments / asset tokenisation programme owner (not publicly named)</t>
+        </is>
+      </c>
+      <c r="E110" s="5" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F110" s="5" t="inlineStr"/>
+      <c r="G110" s="5" t="inlineStr"/>
+      <c r="H110" s="5" t="inlineStr">
+        <is>
+          <t>https://bkam.ma</t>
+        </is>
+      </c>
+      <c r="I110" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>Central Bank of Iraq (CBQ/CBI)</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>IQ</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>Nizar (Hussein/Nasir) - full transliteration varies across sources</t>
+        </is>
+      </c>
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>Governor of the Central Bank of Iraq (appointed Jun 2026, replacing Ali Al-Alaq | oversaw Oct 2026 dinar re-peg to 1,500 IQD/USD)</t>
+        </is>
+      </c>
+      <c r="E111" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F111" s="5" t="inlineStr"/>
+      <c r="G111" s="5" t="inlineStr"/>
+      <c r="H111" s="5" t="inlineStr">
+        <is>
+          <t>https://enterpriseam.com (24 Jun 2026 "Iraq appoints Nizar Hussein as new central bank governor") + en.wikipedia.org/wiki/Central_Bank_of_Iraq ("Nizar Nasir" infobox, Baghdad Today citation)</t>
+        </is>
+      </c>
+      <c r="I111" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="5" t="inlineStr">
+        <is>
+          <t>Central Bank of Iraq</t>
+        </is>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>IQ</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>(position-only)</t>
+        </is>
+      </c>
+      <c r="D112" s="5" t="inlineStr">
+        <is>
+          <t>Deputy Governor for Payments / FX-corridor oversight (dinar-dollar corridor owner | individual not confirmable from accessible sources - corpus-only account, low effort per brief)</t>
+        </is>
+      </c>
+      <c r="E112" s="5" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F112" s="5" t="inlineStr"/>
+      <c r="G112" s="5" t="inlineStr"/>
+      <c r="H112" s="5" t="inlineStr">
+        <is>
+          <t>https://cbi.iq</t>
+        </is>
+      </c>
+      <c r="I112" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>VARA (Dubai)</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>Helal Saeed Almarri</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>Chairman of Executive Board</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F113" s="5" t="inlineStr"/>
+      <c r="G113" s="5" t="inlineStr"/>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>https://www.vara.ae/en/about-vara/</t>
+        </is>
+      </c>
+      <c r="I113" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-10-20 rescued (subagent leg failed to compile)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="5" t="inlineStr">
+        <is>
+          <t>CoinMENA</t>
+        </is>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>Bahrain</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>Talal Tabbaa</t>
+        </is>
+      </c>
+      <c r="D114" s="5" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="E114" s="5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F114" s="5" t="inlineStr"/>
+      <c r="G114" s="5" t="inlineStr"/>
+      <c r="H114" s="5" t="inlineStr">
+        <is>
+          <t>https://www.coinmena.com/en/about-us</t>
+        </is>
+      </c>
+      <c r="I114" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-10-20 rescued</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="5" t="inlineStr">
+        <is>
+          <t>CoinMENA</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>Bahrain</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>Dina Sam'an</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F115" s="5" t="inlineStr"/>
+      <c r="G115" s="5" t="inlineStr"/>
+      <c r="H115" s="5" t="inlineStr">
+        <is>
+          <t>https://www.coinmena.com/en/about-us</t>
+        </is>
+      </c>
+      <c r="I115" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-10-20 rescued</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="5" t="inlineStr">
+        <is>
+          <t>CoinMENA</t>
+        </is>
+      </c>
+      <c r="B116" s="5" t="inlineStr">
+        <is>
+          <t>Bahrain</t>
+        </is>
+      </c>
+      <c r="C116" s="5" t="inlineStr">
+        <is>
+          <t>Yazan Barghuthi</t>
+        </is>
+      </c>
+      <c r="D116" s="5" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="E116" s="5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F116" s="5" t="inlineStr"/>
+      <c r="G116" s="5" t="inlineStr"/>
+      <c r="H116" s="5" t="inlineStr">
+        <is>
+          <t>https://www.coinmena.com/en/about-us</t>
+        </is>
+      </c>
+      <c r="I116" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-10-20 rescued</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="inlineStr">
+        <is>
+          <t>DMCC Crypto Centre</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>H.E. Mansour Mohamed AlMulla</t>
+        </is>
+      </c>
+      <c r="D117" s="5" t="inlineStr">
+        <is>
+          <t>Chairman (also Deputy Group CEO, ADQ)</t>
+        </is>
+      </c>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F117" s="5" t="inlineStr"/>
+      <c r="G117" s="5" t="inlineStr"/>
+      <c r="H117" s="5" t="inlineStr">
+        <is>
+          <t>https://dmcc.ae/latest-news</t>
+        </is>
+      </c>
+      <c r="I117" s="5" t="inlineStr">
+        <is>
+          <t>ENRICHED 2026-10-20 · 2026-10-20 rescued</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="5" t="inlineStr">
+        <is>
+          <t>Zand (UAE digital bank)</t>
+        </is>
+      </c>
+      <c r="B118" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="C118" s="5" t="inlineStr">
+        <is>
+          <t>(position-only)</t>
+        </is>
+      </c>
+      <c r="D118" s="5" t="inlineStr">
+        <is>
+          <t>AI-powered bank partnered with CoinMENA fiat-crypto integration = prospect discovery</t>
+        </is>
+      </c>
+      <c r="E118" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F118" s="5" t="inlineStr"/>
+      <c r="G118" s="5" t="inlineStr"/>
+      <c r="H118" s="5" t="inlineStr">
+        <is>
           <t>https://www.msn.com/en-us/money/other/uae-digital-bank-zand-offers-coinmena-users-seamless-fiat-to-crypto-integration/ar-AA1LnKaq</t>
         </is>
       </c>
-      <c r="I88" s="5" t="inlineStr">
+      <c r="I118" s="5" t="inlineStr">
         <is>
           <t>ENRICHED 2026-10-20 · 2026-09 news</t>
         </is>

</xml_diff>

<commit_message>
EA-50 v2.3: BH-06 Liquid entity-note reconciled (Binance Japan custody arm via Quoine — verify licence entity before outreach); t2 sweep batch consolidated, fold verified complete (54 rows, zero missing)
</commit_message>
<xml_diff>
--- a/ChainSentry-EA50-Master-Targets-20261020.xlsx
+++ b/ChainSentry-EA50-Master-Targets-20261020.xlsx
@@ -7940,7 +7940,11 @@
           <t>tier:T2 conf:medium → Expansion-pool</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr"/>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | ENTITY-NOTE (t2 sweep 21-Oct): Liquid = Binance JAPAN custody arm (Quoine lineage) — "Bahrain regional custody arm" framing reconciled; verify licence entity before outreach</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">

</xml_diff>